<commit_message>
feat: surname dictionary check on all 5 surname fields (alias, emergency, father, mother)
</commit_message>
<xml_diff>
--- a/step1-validation-check.xlsx
+++ b/step1-validation-check.xlsx
@@ -1362,44 +1362,44 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>申請者情報</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>姓</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>苗字チェックアラート</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>候補にない場合アラート</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>未実装</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>苗字辞書データが必要</t>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>486件の日本人姓辞書 + レーベンシュタイン距離(編集距離1-2)でアラート表示</t>
         </is>
       </c>
     </row>
@@ -2012,44 +2012,44 @@
       <c r="H40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>申請者情報</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>姓(別名)</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>苗字チェックアラート</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>候補にない場合アラート</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>未実装</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>苗字辞書データが必要</t>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>486件の日本人姓辞書 + レーベンシュタイン距離(編集距離1-2)でアラート表示</t>
         </is>
       </c>
     </row>

</xml_diff>